<commit_message>
docs: updated sprint status
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_Sprint_Schedule.xlsx
+++ b/docs/development/BantAI_Sprint_Schedule.xlsx
@@ -2181,6 +2181,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
@@ -2263,7 +2264,7 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Resolve Prisma connection issues; commit schema for Android_Users, Contacts, SMS_Messages, Alerts, Protection_Settings, Blocked_Numbers</t>
+          <t>Resolve Prisma connection issues; commit schema for Android_Users, Contacts, SMS_Messages, Alerts, Protection_Settings, Blocked_Numbers — connectivity resolved &amp; core tables done; Contacts, Protection_Settings, Blocked_Numbers carried to S2</t>
         </is>
       </c>
       <c r="D6" s="17" t="n">
@@ -2278,7 +2279,7 @@
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Carried to S2</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2296,7 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Scaffold NestJS project with base module structure and OpenAPI docs</t>
+          <t>Scaffold NestJS project with base module structure and OpenAPI docs — scaffold + modules done; OpenAPI docs pending</t>
         </is>
       </c>
       <c r="D7" s="17" t="n">
@@ -2310,7 +2311,7 @@
       </c>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Carried to S2</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2375,7 @@
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2407,7 @@
       </c>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2439,7 @@
       </c>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2552,7 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>Scaffold Next.js project</t>
+          <t>Scaffold React + Vite project</t>
         </is>
       </c>
       <c r="D15" s="17" t="n">
@@ -2630,7 +2631,7 @@
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2663,7 @@
       </c>
       <c r="G18" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2695,7 @@
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ai): label scheme refinement, softmax routing with gap check
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_Sprint_Schedule.xlsx
+++ b/docs/development/BantAI_Sprint_Schedule.xlsx
@@ -2727,7 +2727,7 @@
       </c>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>Implement softmax classification head (Likely Smishing / Suspicious / Unknown)</t>
+          <t>Implement softmax classification head (Ham / Spam / Scam)</t>
         </is>
       </c>
       <c r="D22" s="17" t="n">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(mobile): wire Campaigns screens to backend, sync WBS/DEV_LOG
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_Sprint_Schedule.xlsx
+++ b/docs/development/BantAI_Sprint_Schedule.xlsx
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C36" s="16" t="inlineStr">
         <is>
-          <t>Build Alert Screen and Suspicious Alert Screen</t>
+          <t>Build Alert Screen and Suspicious Alert Screen — UI built (fully navigable), but running on hardcoded mock data; no backend endpoint to list a user's alerts exists yet</t>
         </is>
       </c>
       <c r="D36" s="17" t="n">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="G36" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Build Campaign Screen, Active/Inactive Campaign Modal/Screen</t>
+          <t>Build Campaign Screen, Active/Inactive Campaign Modal/Screen — Active screen wired to real GET /campaigns and GET /campaigns/:id; Inactive/Modal still on a not-available state, blocked on a backend filter for inactive clusters</t>
         </is>
       </c>
       <c r="D37" s="17" t="n">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="G37" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>
-          <t>Build Notifications: Threat Alert, Weekly Report, Smishing Alert, Weekly Alert</t>
+          <t>Build Notifications: Threat Alert, Weekly Report, Smishing Alert, Weekly Alert — built as one tabbed screen (Threat alerts / Weekly digest); toggle state is real (DataStore), preview content still static</t>
         </is>
       </c>
       <c r="D38" s="17" t="n">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="G38" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>Build Settings: Scam Awareness Tips Screen and Tip Details Screen</t>
+          <t>Build Settings: Scam Awareness Tips Screen and Tip Details Screen — UI built and navigable by real tip ID, but content is hardcoded; no backend endpoint exists for tips yet</t>
         </is>
       </c>
       <c r="D39" s="17" t="n">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="G39" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(mobile): resolve merge-duplicated alerts/campaigns code, sync WBS/sprint docs
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_Sprint_Schedule.xlsx
+++ b/docs/development/BantAI_Sprint_Schedule.xlsx
@@ -660,7 +660,7 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>As of Jul 20, 2026: Sprint 1 complete, Sprint 2 in progress.</t>
+          <t>As of Aug 7, 2026: Sprints 1-3 complete, Sprint 4 in progress.</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="J7" s="20" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="J8" s="21" t="inlineStr">
         <is>
-          <t>Upcoming</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="J9" s="21" t="inlineStr">
         <is>
-          <t>Upcoming</t>
+          <t>Current</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Sprint 2
-(Current)</t>
+(Completed)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1478,7 +1478,7 @@
       <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Sprint 3
-(Upcoming)</t>
+(Completed)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1622,7 +1622,7 @@
       <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Sprint 4
-(Upcoming)</t>
+(Current)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Resolve Prisma connection issues; commit schema for Android_Users, Contacts, SMS_Messages, Alerts, Protection_Settings, Blocked_Numbers — connectivity resolved &amp; core tables done; Contacts, Protection_Settings, Blocked_Numbers carried to S2</t>
+          <t>Resolve Prisma connection issues; commit schema for Android_Users, Contacts, SMS_Messages, Alerts, Blocked_Numbers — all resolved; Contacts + Blocked_Numbers landed in the Sprint 3 schema. Protection_Settings was never modeled as its own table (no dedicated notification-preference table exists in Prisma).</t>
         </is>
       </c>
       <c r="D6" s="17" t="n">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Carried to S2</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Scaffold NestJS project with base module structure and OpenAPI docs — scaffold + modules done; OpenAPI docs pending</t>
+          <t>Scaffold NestJS project with base module structure — done. OpenAPI/Swagger UI was never added (no @nestjs/swagger dependency); API is documented manually instead via docs/api/*.md files.</t>
         </is>
       </c>
       <c r="D7" s="17" t="n">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>Carried to S2</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="G29" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="G30" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="G31" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
       </c>
       <c r="G32" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3142,7 @@
       </c>
       <c r="G33" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="G34" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3206,7 @@
       </c>
       <c r="G35" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C36" s="16" t="inlineStr">
         <is>
-          <t>Build Alert Screen and Suspicious Alert Screen — UI built (fully navigable), but running on hardcoded mock data; no backend endpoint to list a user's alerts exists yet</t>
+          <t>Build Alert Screen and Suspicious Alert Screen — wired to real GET /sms/alerts and GET /sms/:messageId/indicators; committed and merged to develop.</t>
         </is>
       </c>
       <c r="D36" s="17" t="n">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="G36" s="18" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Build Campaign Screen, Active/Inactive Campaign Modal/Screen — Active screen wired to real GET /campaigns and GET /campaigns/:id; Inactive/Modal still on a not-available state, blocked on a backend filter for inactive clusters</t>
+          <t>Build Campaign Screen, Active/Inactive Campaign Modal/Screen — both Active and Inactive wired to real GET /campaigns, GET /campaigns/inactive, GET /campaigns/:id; committed and merged.</t>
         </is>
       </c>
       <c r="D37" s="17" t="n">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="G37" s="18" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>
-          <t>Build Notifications: Threat Alert, Weekly Report, Smishing Alert, Weekly Alert — built as one tabbed screen (Threat alerts / Weekly digest); toggle state is real (DataStore), preview content still static</t>
+          <t>Build Notifications: Threat Alert, Weekly Report, Smishing Alert, Weekly Alert — Threat alerts tab wired to real GET /sms/alerts; Weekly digest tab intentionally stays a labeled preview (no backend weekly-report generation exists — a separate future feature, not a Sprint 3 blocker).</t>
         </is>
       </c>
       <c r="D38" s="17" t="n">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="G38" s="18" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>Build Settings: Scam Awareness Tips Screen and Tip Details Screen — UI built and navigable by real tip ID, but content is hardcoded; no backend endpoint exists for tips yet</t>
+          <t>Build Settings: Scam Awareness Tips Screen and Tip Details Screen — ScamAwarenessViewModel derives per-user relevant tips from real GET /sms/alerts data; tip educational content itself is static reference text by design.</t>
         </is>
       </c>
       <c r="D39" s="17" t="n">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="G39" s="18" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="G40" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="G41" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Build automated retraining workflow (snapshot, AdamW fine-tune, reservoir update, McNemar/F1 gate)</t>
+          <t>Build automated retraining workflow (snapshot, AdamW fine-tune, reservoir update, McNemar/promotion gate) — reservoir sampling + McNemar/F1-floor promotion gate logic done in ai/retraining/; end-to-end pipeline wiring blocked on UserReports (row above).</t>
         </is>
       </c>
       <c r="D45" s="17" t="n">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="G45" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="G46" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="G47" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3607,7 @@
       </c>
       <c r="C48" s="16" t="inlineStr">
         <is>
-          <t>Build Compose Message Screen and Unknown Filter Screen</t>
+          <t>Build Compose Message Screen and Unknown Filter Screen — Compose Message fully done (real SmsManager send, drafts, outbox/sent/failed states); Unknown Filter screen not started (no UNKNOWN case in MessageFilter).</t>
         </is>
       </c>
       <c r="D48" s="17" t="n">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="G48" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="C49" s="16" t="inlineStr">
         <is>
-          <t>Build AI Message Summary display</t>
+          <t>Build AI Message Summary display — AISummaryBottomSheet wired to a real suspicious/unknown trigger signal, but verdict text and confidence % are still hardcoded; no mobile client or backend proxy for the AI service's POST /summarize yet.</t>
         </is>
       </c>
       <c r="D49" s="17" t="n">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="G49" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="C50" s="16" t="inlineStr">
         <is>
-          <t>Build Settings: Blocked Numbers Screen</t>
+          <t>Build Settings: Blocked Numbers Screen — screen fully built (list, unblock, confirm dialog) but purely device-local via Android's BlockedNumberContract; not synced to the backend's BlockedNumber table.</t>
         </is>
       </c>
       <c r="D50" s="17" t="n">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="G50" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="G51" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="G52" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3782,7 +3782,7 @@
       </c>
       <c r="G53" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3846,7 @@
       </c>
       <c r="G55" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: close Sprint 4, sync WBS/DEV_LOG trackers, fix stale xlsx entries
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_Sprint_Schedule.xlsx
+++ b/docs/development/BantAI_Sprint_Schedule.xlsx
@@ -661,7 +661,7 @@
     <row r="3">
       <c r="A3" s="35" t="inlineStr">
         <is>
-          <t>As of Aug 16, 2026: Sprints 1-3 complete. Sprint 4 Backend/AI-ML/Web Dashboard tracks complete (Web is UI-complete on mock data, not yet backend-wired); Mobile track and the cross-track retraining integration test still in progress. Sprint 5 groundwork already underway on Track B.</t>
+          <t>As of Aug 18, 2026: Sprints 1-4 complete, including the Sprint 4 retro. Known limitation carried forward, not a Sprint 4 blocker: the mobile app has no deployed backend yet -- Alerts/Campaigns (and every other live-API screen) only work while the phone is tethered to a dev laptop (adb reverse tcp:3000 or the 10.0.2.2 emulator loopback); real deployment is explicitly Sprint 6 scope. Sprint 5 now current -- threshold re-calibration (5.3.6) and indicator-tag polish already underway on Track B.</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="J9" s="42" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="J10" s="42" t="inlineStr">
         <is>
-          <t>Upcoming</t>
+          <t>Current</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1" s="33">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -3513,7 +3512,7 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Build automated retraining workflow (snapshot, AdamW fine-tune, reservoir update, McNemar/promotion gate) — reservoir sampling + McNemar/F1-floor promotion gate logic done in ai/retraining/; UserReports table now exists (Track A), but ai/retraining/reports.py has no DatabaseReportSource wired to it yet, and no real GPU fine-tune has run.</t>
+          <t>Build automated retraining workflow (snapshot, AdamW fine-tune, reservoir update, McNemar/promotion gate) — complete end to end. DatabaseReportSource now reads validated reports live from GET /api/reports; first real GPU fine-tune ran 2026-08-17 (Colab T4), macro-F1 0.9520-&gt;0.9648, gate says promote. Not promoted yet, pending adviser sign-off (swap would invalidate Sprint 5 threshold calibration). Merged to develop via PR #52.</t>
         </is>
       </c>
       <c r="D45" s="8" t="n">
@@ -3528,7 +3527,7 @@
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3544,7 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Build campaign evolution tracking logic</t>
+          <t>Build campaign evolution tracking logic -- campaign_evolution.py (386 lines, pure module) + scripts/track_campaign_evolution.py (CLI) + 30 tests. Compares HDBSCAN snapshots for new/dropped/grown/merged/fragmented campaigns.</t>
         </is>
       </c>
       <c r="D46" s="8" t="n">
@@ -3560,7 +3559,7 @@
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3960,7 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Polish SHAP indicator tag dictionary based on observed outputs</t>
+          <t>Polish SHAP indicator tag dictionary based on observed outputs -- measured via analyze_indicator_coverage.py against every labeled Spam/Scam row; Scam zero-tag rate 48.6% -&gt; 40.0% after adding Tagalog online-betting vocabulary and a phishing phrasing gap. Merged via PR #54.</t>
         </is>
       </c>
       <c r="D59" s="8" t="n">
@@ -3976,7 +3975,7 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(mobile): wire Terms/Allow-Access screens, fix phone normalization and nav badge, redesign profile screen (WBS 5.3.9)
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_Sprint_Schedule.xlsx
+++ b/docs/development/BantAI_Sprint_Schedule.xlsx
@@ -4024,7 +4024,7 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>UI polish based on internal dogfooding</t>
+          <t>UI polish based on internal dogfooding -- ran the real flow live, fixed real bugs found by doing so (orphaned Terms/Allow-Access screens, phone number normalization, hardcoded nav badge, dead back button), redesigned profile screen + added app-wide screen transitions and tab cross-fade animation.</t>
         </is>
       </c>
       <c r="D61" s="8" t="n">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: close WBS 5.3.8/5.4.3, log Maxene's AI holdout merge, sync xlsx trackers
</commit_message>
<xml_diff>
--- a/docs/development/BantAI_Sprint_Schedule.xlsx
+++ b/docs/development/BantAI_Sprint_Schedule.xlsx
@@ -3992,7 +3992,7 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Bug bash: unusual sender formats, mixed-language edge cases, low-end device performance</t>
+          <t>Bug bash: unusual sender formats, mixed-language edge cases, low-end device performance -- Fixed a real SmsReceiver crash (empty PDU array), blank-sender bugs, a negative-clock-skew display bug, load races in 3 ViewModels, phone-validation, and an onboarding IME-scroll issue. Also caught+fixed live: an EMUI floating-window gesture crash. Live-verified on a physical device except the SmsReceiver empty-PDU guard (code-review only). Merged via PR #59, 2026-08-20.</t>
         </is>
       </c>
       <c r="D60" s="8" t="n">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4280,7 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>False positive / false negative confusion matrix review</t>
+          <t>False positive / false negative confusion matrix review -- Maxene: permanent 20% held-out split carved (create_holdout_set.py, 3,236 rows) + first eval run (evaluate_holdout.py, macro-F1 0.95), but that run is explicitly caveated as not a clean test since the deployed model was trained before the split existed. Real result needs the next model trained after 2026-08-18. Merged via PR #56/#58, 2026-08-20.</t>
         </is>
       </c>
       <c r="D69" s="8" t="n">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>

</xml_diff>